<commit_message>
0.8.7 ground and tact polishing
+ добавил технике урон от арты
</commit_message>
<xml_diff>
--- a/tactical_battle_log.xlsx
+++ b/tactical_battle_log.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tactical_log" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ground_log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="player_plan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="enemy_plan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,7 +517,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46155.41666666666</v>
+        <v>46155.5</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -523,22 +525,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I2" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -547,13 +549,13 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="M2" t="n">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -561,27 +563,27 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>46155.5</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B1 против B1</t>
+          <t>B2 против B2</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H3" t="n">
         <v>56</v>
@@ -596,67 +598,16 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="M3" t="n">
-        <v>88</v>
+        <v>24</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
         <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-05-13 14:00:00</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>B2 рубиццо</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>32</v>
-      </c>
-      <c r="I4" t="n">
-        <v>32</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -670,7 +621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -766,7 +717,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-13 10:00:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -774,59 +725,39 @@
           <t>blue</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>BLU_2</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>mlrs</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>72</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>RED_5</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>36</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>18</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>разгром</t>
-        </is>
+          <t>art_air_fire</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -835,7 +766,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-13 10:15:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -843,59 +774,39 @@
           <t>blue</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>BLU_2</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>mlrs</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>70</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>5</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>RED_6</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>36</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
+          <t>RED_5</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>9</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>победа</t>
-        </is>
+          <t>art_air_fire</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -904,7 +815,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-13 10:15:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -912,59 +823,39 @@
           <t>blue</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>BLU_3</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>mlrs</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>72</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>RED_5</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>18</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
+          <t>RED_3</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>победа</t>
-        </is>
+          <t>art_air_fire</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -973,7 +864,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-13 10:30:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -981,59 +872,39 @@
           <t>blue</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>BLU_3</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>mlrs</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>72</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>RED_6</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>27</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
+          <t>RED_1</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
         <v>5</v>
       </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>засада</t>
-        </is>
+          <t>art_air_fire</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1042,7 +913,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-13 10:45:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1052,7 +923,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>BLU_3</t>
+          <t>BLU_6</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1061,20 +932,20 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>RED_6</t>
+          <t>RED_4</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1083,13 +954,13 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -1101,7 +972,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>поражение</t>
+          <t>засада</t>
         </is>
       </c>
     </row>
@@ -1111,7 +982,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-13 11:00:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1121,7 +992,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BLU_4</t>
+          <t>BLU_1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1130,7 +1001,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1143,7 +1014,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>RED_6</t>
+          <t>RED_2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1152,13 +1023,13 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
@@ -1180,7 +1051,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-13 10:30:00</t>
+          <t>2026-05-13 12:15:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1190,7 +1061,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BLU_2</t>
+          <t>BLU_6</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1199,20 +1070,20 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>65</v>
+        <v>29</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>RED_5</t>
+          <t>RED_1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1221,13 +1092,13 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>13</v>
+        <v>79</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -1239,7 +1110,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>поражение</t>
+          <t>засада</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1120,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-13 10:00:00</t>
+          <t>2026-05-13 12:30:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1259,7 +1130,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>BLU_5</t>
+          <t>BLU_1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1268,7 +1139,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -1281,7 +1152,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>RED_4</t>
+          <t>RED_1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1290,13 +1161,13 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -1308,7 +1179,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>победа</t>
+          <t>разгром</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1189,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-13 11:15:00</t>
+          <t>2026-05-13 12:15:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1328,7 +1199,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>BLU_4</t>
+          <t>BLU_3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1337,20 +1208,20 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>RED_4</t>
+          <t>RED_2</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1359,13 +1230,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1387,7 +1258,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-13 11:30:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1395,59 +1266,41 @@
           <t>blue</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>BLU_4</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>cannon</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>32</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>RED_6</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>16</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>art_air_fire</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
         <v>2</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>RED_4</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L11" t="n">
-        <v>32</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
-        <v>2</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>победа</t>
-        </is>
       </c>
     </row>
     <row r="12">
@@ -1456,7 +1309,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-05-13 11:15:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1464,59 +1317,41 @@
           <t>blue</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>BLU_5</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>cannon</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>36</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>0</v>
       </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>RED_6</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L12" t="n">
-        <v>17</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0</v>
-      </c>
+          <t>RED_5</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
+        <v>16</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>art_air_fire</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
         <v>2</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>победа</t>
-        </is>
       </c>
     </row>
     <row r="13">
@@ -1525,7 +1360,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-05-13 11:00:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1533,59 +1368,41 @@
           <t>blue</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>BLU_3</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>cannon</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>63</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>4</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>RED_1</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>72</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
+          <t>RED_4</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>ничья</t>
-        </is>
+          <t>art_air_fire</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1594,7 +1411,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-13 11:45:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1604,7 +1421,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BLU_4</t>
+          <t>BLU_1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1613,47 +1430,47 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>RED_4</t>
+          <t>RED_2</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>mech</t>
         </is>
       </c>
       <c r="L14" t="n">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
+          <t>inf_attacks_mech</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>ничья</t>
+          <t>поражение</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1480,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-13 10:45:00</t>
+          <t>2026-05-13 12:15:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1673,7 +1490,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BLU_2</t>
+          <t>BLU_5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1682,13 +1499,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -1700,14 +1517,14 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>mech</t>
         </is>
       </c>
       <c r="L15" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -1717,12 +1534,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
+          <t>inf_attacks_mech</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>поражение</t>
+          <t>ничья</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1549,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-13 11:30:00</t>
+          <t>2026-05-13 12:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1742,7 +1559,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>BLU_5</t>
+          <t>BLU_2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1751,13 +1568,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -1773,13 +1590,13 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
@@ -1791,86 +1608,86 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>поражение</t>
+          <t>победа</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-05-13 12:00:00</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BLU_6</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>37</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>RED_4</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>mech</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>31</v>
+      </c>
+      <c r="M17" t="n">
         <v>2</v>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026-05-13 12:00:00</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>blue</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>BLU_4</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>36</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>3</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>RED_4</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L17" t="n">
-        <v>36</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0</v>
-      </c>
       <c r="N17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
+          <t>inf_attacks_mech</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ничья</t>
+          <t>победа</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-13 12:00:00</t>
+          <t>2026-05-13 12:15:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1880,7 +1697,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>BLU_1</t>
+          <t>BLU_6</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1889,20 +1706,20 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>RED_1</t>
+          <t>RED_3</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1911,13 +1728,13 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
@@ -1929,17 +1746,17 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>поражение</t>
+          <t>засада</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-13 12:00:00</t>
+          <t>2026-05-13 12:30:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1949,7 +1766,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>BLU_2</t>
+          <t>BLU_5</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1958,7 +1775,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1971,44 +1788,44 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>RED_3</t>
+          <t>RED_7</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>arm</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N19" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
+          <t>inf_attacks_armor</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>разгром</t>
+          <t>anti_armor_attack</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-13 12:15:00</t>
+          <t>2026-05-13 12:45:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2018,7 +1835,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BLU_4</t>
+          <t>BLU_1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2027,57 +1844,57 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>RED_5</t>
+          <t>RED_7</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>arm</t>
         </is>
       </c>
       <c r="L20" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
+          <t>inf_attacks_armor</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>поражение</t>
+          <t>anti_armor_attack</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-13 12:30:00</t>
+          <t>2026-05-13 13:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2087,7 +1904,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>BLU_3</t>
+          <t>BLU_1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2096,101 +1913,101 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>RED_5</t>
+          <t>RED_4</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>mech</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
+          <t>inf_attacks_mech</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>разгром</t>
+          <t>засада</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-05-13 13:15:00</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>BLU_3</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>54</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
         <v>2</v>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>2026-05-13 12:45:00</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>blue</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>BLU_3</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>59</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" t="n">
-        <v>28</v>
-      </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>RED_6</t>
+          <t>RED_4</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>mech</t>
         </is>
       </c>
       <c r="L22" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" t="n">
         <v>0</v>
@@ -2200,22 +2017,22 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
+          <t>inf_attacks_mech</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>засада</t>
+          <t>поражение</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-13 12:15:00</t>
+          <t>2026-05-13 13:30:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2225,7 +2042,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>BLU_5</t>
+          <t>BLU_3</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2234,57 +2051,57 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>RED_1</t>
+          <t>RED_4</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>mech</t>
         </is>
       </c>
       <c r="L23" t="n">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
+          <t>inf_attacks_mech</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>ничья</t>
+          <t>разгром</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-05-13 12:15:00</t>
+          <t>2026-05-13 13:15:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2294,7 +2111,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>BLU_6</t>
+          <t>BLU_1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2303,254 +2120,1671 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
+        <v>4</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>RED_2</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>mech</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>84</v>
+      </c>
+      <c r="M24" t="n">
         <v>3</v>
       </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>RED_4</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L24" t="n">
-        <v>34</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
       <c r="N24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>inf_attacks_inf</t>
+          <t>inf_attacks_mech</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>ничья</t>
+          <t>поражение</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-05-13 12:15:00</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>BLU_2</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>83</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>RED_5</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>mech</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>26</v>
+      </c>
+      <c r="M25" t="n">
+        <v>2</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>inf_attacks_mech</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>ничья</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>tactical_buttle_num</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>temp_unit_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source_level</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>source_uid</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>slice_label</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>split_basis</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>soldiers</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>company_uids</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>platoon_uids</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>squad_uids</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>unit_role</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BLU_1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>B1-C3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>B1-C3-PART1[B1-C3-P1..B1-C3-P3]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>84</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>B1-C3</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>B1-C3-P1,B1-C3-P3</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>B1-C3-P1-S1,B1-C3-P1-S2,B1-C3-P1-S3,B1-C3-P3-S1,B1-C3-P3-S2,B1-C3-P3-S3</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BLU_2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>B1-C2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B1-C2-PART1[B1-C2-P1..B1-C2-P3]</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>84</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>B1-C2</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>B1-C2-P1,B1-C2-P3</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>B1-C2-P1-S1,B1-C2-P1-S2,B1-C2-P1-S3,B1-C2-P3-S1,B1-C2-P3-S2,B1-C2-P3-S3</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BLU_3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>B1-C1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>B1-C1-PART1[B1-C1-P1..B1-C1-P3]</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>84</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>B1-C1</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>B1-C1-P1,B1-C1-P3</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>B1-C1-P1-S1,B1-C1-P1-S2,B1-C1-P1-S3,B1-C1-P3-S1,B1-C1-P3-S2,B1-C1-P3-S3</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BLU_4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B1-C3-P2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>B1-C3-PART2[B1-C3-P2..B1-C3-P2]</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>42</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>B1-C3</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>B1-C3-P2</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>B1-C3-P2-S1,B1-C3-P2-S2,B1-C3-P2-S3</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BLU_5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B1-C2-P2</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>B1-C2-PART2[B1-C2-P2..B1-C2-P2]</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>42</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>B1-C2</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>B1-C2-P2</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>B1-C2-P2-S1,B1-C2-P2-S2,B1-C2-P2-S3</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BLU_6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B1-C1-P2</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>B1-C1-PART2[B1-C1-P2..B1-C1-P2]</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>42</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>B1-C1</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>B1-C1-P2</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>B1-C1-P2-S1,B1-C1-P2-S2,B1-C1-P2-S3</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BLU_1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B1-C3</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B1-C3-PART1[B1-C3-P1..B1-C3-P3]</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>84</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>B1-C3</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>B1-C3-P1,B1-C3-P3</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>B1-C3-P1-S1,B1-C3-P1-S2,B1-C3-P1-S3,B1-C3-P3-S1,B1-C3-P3-S2,B1-C3-P3-S3</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BLU_2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B1-C2</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B1-C2-PART1[B1-C2-P1..B1-C2-P3]</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>84</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>B1-C2</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>B1-C2-P1,B1-C2-P3</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>B1-C2-P1-S1,B1-C2-P1-S2,B1-C2-P1-S3,B1-C2-P3-S1,B1-C2-P3-S2,B1-C2-P3-S3</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BLU_3</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B1-C1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B1-C1-PART2[B1-C1-P2..B1-C1-P3]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>54</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>B1-C1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>B1-C1-P2,B1-C1-P3</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>B1-C1-P2-S1,B1-C1-P2-S2,B1-C1-P2-S3,B1-C1-P3-S1,B1-C1-P3-S2,B1-C1-P3-S3</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BLU_4</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>B1-C3-P2</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>B1-C3-PART2[B1-C3-P2..B1-C3-P2]</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>42</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>B1-C3</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>B1-C3-P2</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>B1-C3-P2-S1,B1-C3-P2-S2,B1-C3-P2-S3</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BLU_5</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>B1-C2-P2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>B1-C2-PART2[B1-C2-P2..B1-C2-P2]</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>42</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>B1-C2</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>B1-C2-P2</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>B1-C2-P2-S1,B1-C2-P2-S2,B1-C2-P2-S3</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BLU_6</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>B1-C1-P1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>B1-C1-PART1[B1-C1-P1..B1-C1-P1]</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>37</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>B1-C1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>B1-C1-P1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>B1-C1-P1-S1,B1-C1-P1-S2,B1-C1-P1-S3</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>tactical_buttle_num</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>temp_unit_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source_level</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>source_uid</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>slice_label</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>split_basis</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>soldiers</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>company_uids</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>platoon_uids</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>squad_uids</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>unit_role</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>unit_role_armor</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>assigned_armor</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>source_armor_uids</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RED_1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>B1-C3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>B1-C3-PART1[B1-C3-P1..B1-C3-P3]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>84</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>B1-C3</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>B1-C3-P1,B1-C3-P3</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>B1-C3-P1-S1,B1-C3-P1-S2,B1-C3-P1-S3,B1-C3-P3-S1,B1-C3-P3-S2,B1-C3-P3-S3</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RED_2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>B1-C2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B1-C2-PART1[B1-C2-P1..B1-C2-P3]</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>84</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>B1-C2</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>B1-C2-P1,B1-C2-P3</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>B1-C2-P1-S1,B1-C2-P1-S2,B1-C2-P1-S3,B1-C2-P3-S1,B1-C2-P3-S2,B1-C2-P3-S3</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RED_3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>B1-C1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>B1-C1-PART1[B1-C1-P1..B1-C1-P3]</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>84</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>B1-C1</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>B1-C1-P1,B1-C1-P3</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>B1-C1-P1-S1,B1-C1-P1-S2,B1-C1-P1-S3,B1-C1-P3-S1,B1-C1-P3-S2,B1-C1-P3-S3</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RED_4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B1-C3-P2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>B1-C3-PART2[B1-C3-P2..B1-C3-P2]</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>42</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>B1-C3</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>B1-C3-P2</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>B1-C3-P2-S1,B1-C3-P2-S2,B1-C3-P2-S3</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RED_5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>B1-C2-P2</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>B1-C2-PART2[B1-C2-P2..B1-C2-P2]</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>42</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>B1-C2</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>B1-C2-P2</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>B1-C2-P2-S1,B1-C2-P2-S2,B1-C2-P2-S3</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>RED_6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B1-C1-P2</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>B1-C1-PART2[B1-C1-P2..B1-C1-P2]</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>42</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>B1-C1</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>B1-C1-P2</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>B1-C1-P2-S1,B1-C1-P2-S2,B1-C1-P2-S3</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RED_1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B3-C3</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B3-C3-PART1[B3-C3-P1..B3-C3-P3]</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>84</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>B3-C3</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>B3-C3-P1,B3-C3-P3</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>B3-C3-P1-S1,B3-C3-P1-S2,B3-C3-P1-S3,B3-C3-P3-S1,B3-C3-P3-S2,B3-C3-P3-S3</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RED_2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B3-C2</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B3-C2-PART1[B3-C2-P1..B3-C2-P3]</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>84</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>B3-C2</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>B3-C2-P1,B3-C2-P3</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>B3-C2-P1-S1,B3-C2-P1-S2,B3-C2-P1-S3,B3-C2-P3-S1,B3-C2-P3-S2,B3-C2-P3-S3</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>mech_attachment</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
         <v>3</v>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2026-05-13 14:00:00</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>blue</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>pc1</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>108</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>b2_c2</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>разгром</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>A28,A29,A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RED_3</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B3-C1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B3-C1-PART1[B3-C1-P1..B3-C1-P3]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>84</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>B3-C1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>B3-C1-P1,B3-C1-P3</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>B3-C1-P1-S1,B3-C1-P1-S2,B3-C1-P1-S3,B3-C1-P3-S1,B3-C1-P3-S2,B3-C1-P3-S3</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>RED_4</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>B3-C3-P2</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>B3-C3-PART2[B3-C3-P2..B3-C3-P2]</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>42</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>B3-C3</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>B3-C3-P2</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>B3-C3-P2-S1,B3-C3-P2-S2,B3-C3-P2-S3</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>mech_attachment</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
         <v>3</v>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2026-05-13 14:00:00</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>blue</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>pc1</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>108</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>b2_c2</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L26" t="n">
-        <v>108</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" t="n">
-        <v>1</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>засада</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>3</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026-05-13 14:00:00</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>blue</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>pc1</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>108</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" t="n">
-        <v>32</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>b2_c2</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L27" t="n">
-        <v>107</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>inf_attacks_inf</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>засада</t>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>A30,A5,A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RED_5</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>B3-C2-P2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>B3-C2-PART2[B3-C2-P2..B3-C2-P2]</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>42</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>B3-C2</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>B3-C2-P2</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>B3-C2-P2-S1,B3-C2-P2-S2,B3-C2-P2-S3</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>mech_attachment</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>A4,A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RED_6</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>B3-C1-P2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>B3-C1-PART2[B3-C1-P2..B3-C1-P2]</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>platoon</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>42</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>B3-C1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>B3-C1-P2</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>B3-C1-P2-S1,B3-C1-P2-S2,B3-C1-P2-S3</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>inf_or_mech</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>mech_attachment</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>A3,A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RED_7</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>RED_7</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>arm</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>20</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>A1,A10,A11,A12,A13,A14,A15,A16,A17,A18,A19,A2,A20,A21,A22,A23,A24,A25,A26,A27</t>
         </is>
       </c>
     </row>

</xml_diff>